<commit_message>
Actualiza KPI Tasa de Instalacion BAF - periodo 2026-08
</commit_message>
<xml_diff>
--- a/periodos/2026-08/reportes/Reporte_Tasa_Instalacion_BAF_2026-08.xlsx
+++ b/periodos/2026-08/reportes/Reporte_Tasa_Instalacion_BAF_2026-08.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\analisis\BBDD\p12_Tasa_Instalacion_BAF_2026-08\periodos\2026-08\reportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFAED390-34CE-45D9-81C3-543405F0F947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CADF2D9B-42DD-4418-9DE9-B11621199546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4375BB14-92FB-4897-896D-B22A6863562C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ADF1982F-1972-4AF9-8C2E-E3CF74272238}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -41,14 +41,14 @@
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
-  <connection id="1" xr16:uid="{52F117A4-E8AE-423A-81D5-DA41311713E7}" name="denominador_maestro_ventas" type="6" refreshedVersion="8" background="1" saveData="1">
+  <connection id="1" xr16:uid="{95E707BC-C7C1-44F6-8235-E5A9E7411A0B}" name="denominador_maestro_ventas" type="6" refreshedVersion="8" background="1" saveData="1">
     <textPr prompt="0" sourceFile="C:\analisis\BBDD\p12_Tasa_Instalacion_BAF_2026-08\periodos\2026-08\datos\denominador_maestro_ventas.csv" decimal="," thousands="." semicolon="1">
       <textFields>
         <textField/>
       </textFields>
     </textPr>
   </connection>
-  <connection id="2" xr16:uid="{12DA9F16-DBEE-4AF7-90FF-250E44366F48}" name="numerador_filtrado" type="6" refreshedVersion="8" background="1" saveData="1">
+  <connection id="2" xr16:uid="{81DEA760-D33F-4833-9ECC-5B9D5134769E}" name="numerador_filtrado" type="6" refreshedVersion="8" background="1" saveData="1">
     <textPr prompt="0" sourceFile="C:\analisis\BBDD\p12_Tasa_Instalacion_BAF_2026-08\periodos\2026-08\datos\numerador_filtrado.csv" decimal="," thousands="." semicolon="1">
       <textFields>
         <textField/>
@@ -278,7 +278,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-EF10-4D47-BFD3-39DFB837687D}"/>
+              <c16:uniqueId val="{00000001-D4D0-406A-8F53-40BFB5AC4B62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -306,7 +306,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-EF10-4D47-BFD3-39DFB837687D}"/>
+              <c16:uniqueId val="{00000002-D4D0-406A-8F53-40BFB5AC4B62}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -319,11 +319,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="1432324063"/>
-        <c:axId val="1326142191"/>
+        <c:axId val="1625124096"/>
+        <c:axId val="1611325360"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1432324063"/>
+        <c:axId val="1625124096"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -333,7 +333,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1326142191"/>
+        <c:crossAx val="1611325360"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -341,7 +341,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1326142191"/>
+        <c:axId val="1611325360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -352,7 +352,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1432324063"/>
+        <c:crossAx val="1625124096"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -400,7 +400,7 @@
         <xdr:cNvPr id="2" name="Gráfico 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC889BA6-3904-0334-680C-CD54BD7181A2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8117F603-15BC-4A1D-9C49-7A4028580A1A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -422,11 +422,11 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatosExternos_1" connectionId="2" xr16:uid="{5AA457A4-0BBF-4123-821B-9CFA7E51EEEB}" autoFormatId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatosExternos_1" connectionId="2" xr16:uid="{82EB585D-F463-4047-8B6C-6DB465E8A6A5}" autoFormatId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatosExternos_1" connectionId="1" xr16:uid="{4F3617E4-D8F9-42D3-B78F-4B2B828570D9}" autoFormatId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatosExternos_1" connectionId="1" xr16:uid="{66A8D0F0-4227-434D-9F3E-F6FAAFE8F3A4}" autoFormatId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -745,7 +745,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63F454A6-6686-47C0-B22E-74C09F25C94D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CF2D0D3-DF70-4E68-AAA0-A2892CF57614}">
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -847,7 +847,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8264DBEF-7650-4F23-B68E-C60FEDBEB372}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CD0614-2727-4D28-A116-2B5804F63E8B}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -858,7 +858,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DA31F82-406C-4057-B82F-32E772170527}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D376F7-1D9E-425F-8FFF-6405DC390B97}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>